<commit_message>
Add cost delta to break-even point in Excel
</commit_message>
<xml_diff>
--- a/stock_portfolio_tracker.xlsx
+++ b/stock_portfolio_tracker.xlsx
@@ -615,7 +615,7 @@
     </row>
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="7">
-        <f>IF(COUNTA(B10:B104)=0,"","⚖️ 盈亏平衡点: $"&amp;TEXT(G10-I10/H10,"#,##0.00"))</f>
+        <f>IF(COUNTA(B10:B104)=0,"","⚖️ 盈亏平衡点: $"&amp;TEXT(G10-IFERROR(I10/H10,0),"#,##0.00")&amp;"  (差价: $"&amp;TEXT(-IFERROR(I10/H10,0),"#,##0.00")&amp;")")</f>
         <v/>
       </c>
     </row>
@@ -669,17 +669,17 @@
       </c>
       <c r="B10" s="10" t="inlineStr">
         <is>
-          <t>卖出</t>
+          <t>买入</t>
         </is>
       </c>
       <c r="C10" s="10" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D10" s="10" t="n">
-        <v>389.09</v>
+        <v>372</v>
       </c>
       <c r="E10" s="10" t="n">
-        <v>0.03</v>
+        <v>0</v>
       </c>
       <c r="F10" s="11">
         <f>IF(B10="卖出",IF(H11&lt;=0,"",(D10-G11)*C10-E10),"")</f>
@@ -701,22 +701,22 @@
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B11" s="10" t="inlineStr">
         <is>
-          <t>买入</t>
+          <t>卖出</t>
         </is>
       </c>
       <c r="C11" s="10" t="n">
         <v>4</v>
       </c>
       <c r="D11" s="10" t="n">
-        <v>386</v>
+        <v>377</v>
       </c>
       <c r="E11" s="10" t="n">
-        <v>0</v>
+        <v>0.03</v>
       </c>
       <c r="F11" s="11">
         <f>IF(B11="卖出",IF(H12&lt;=0,"",(D11-G12)*C11-E11),"")</f>
@@ -738,22 +738,22 @@
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B12" s="10" t="inlineStr">
         <is>
-          <t>卖出</t>
+          <t>买入</t>
         </is>
       </c>
       <c r="C12" s="10" t="n">
         <v>4</v>
       </c>
       <c r="D12" s="10" t="n">
-        <v>399</v>
+        <v>376</v>
       </c>
       <c r="E12" s="10" t="n">
-        <v>0.03</v>
+        <v>0</v>
       </c>
       <c r="F12" s="11">
         <f>IF(B12="卖出",IF(H13&lt;=0,"",(D12-G13)*C12-E12),"")</f>
@@ -775,22 +775,22 @@
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B13" s="10" t="inlineStr">
         <is>
-          <t>买入</t>
+          <t>卖出</t>
         </is>
       </c>
       <c r="C13" s="10" t="n">
         <v>4</v>
       </c>
       <c r="D13" s="10" t="n">
-        <v>392</v>
+        <v>389.09</v>
       </c>
       <c r="E13" s="10" t="n">
-        <v>0</v>
+        <v>0.03</v>
       </c>
       <c r="F13" s="11">
         <f>IF(B13="卖出",IF(H14&lt;=0,"",(D13-G14)*C13-E13),"")</f>
@@ -812,22 +812,22 @@
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B14" s="10" t="inlineStr">
         <is>
-          <t>卖出</t>
+          <t>买入</t>
         </is>
       </c>
       <c r="C14" s="10" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D14" s="10" t="n">
-        <v>397</v>
+        <v>386</v>
       </c>
       <c r="E14" s="10" t="n">
-        <v>0.02</v>
+        <v>0</v>
       </c>
       <c r="F14" s="11">
         <f>IF(B14="卖出",IF(H15&lt;=0,"",(D14-G15)*C14-E14),"")</f>
@@ -849,22 +849,22 @@
     <row r="15">
       <c r="A15" s="9" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B15" s="10" t="inlineStr">
         <is>
-          <t>买入</t>
+          <t>卖出</t>
         </is>
       </c>
       <c r="C15" s="10" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D15" s="10" t="n">
-        <v>392.5</v>
+        <v>399</v>
       </c>
       <c r="E15" s="10" t="n">
-        <v>0</v>
+        <v>0.03</v>
       </c>
       <c r="F15" s="11">
         <f>IF(B15="卖出",IF(H16&lt;=0,"",(D15-G16)*C15-E15),"")</f>
@@ -895,10 +895,10 @@
         </is>
       </c>
       <c r="C16" s="10" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D16" s="10" t="n">
-        <v>396.27</v>
+        <v>392</v>
       </c>
       <c r="E16" s="10" t="n">
         <v>0</v>
@@ -928,17 +928,17 @@
       </c>
       <c r="B17" s="10" t="inlineStr">
         <is>
-          <t>买入</t>
+          <t>卖出</t>
         </is>
       </c>
       <c r="C17" s="10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D17" s="10" t="n">
-        <v>398.6828</v>
+        <v>397</v>
       </c>
       <c r="E17" s="10" t="n">
-        <v>0</v>
+        <v>0.02</v>
       </c>
       <c r="F17" s="11">
         <f>IF(B17="卖出",IF(H18&lt;=0,"",(D17-G18)*C17-E17),"")</f>
@@ -969,10 +969,10 @@
         </is>
       </c>
       <c r="C18" s="10" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D18" s="10" t="n">
-        <v>401.385</v>
+        <v>392.5</v>
       </c>
       <c r="E18" s="10" t="n">
         <v>0</v>
@@ -997,19 +997,19 @@
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
         <is>
-          <t>2026-01-02</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B19" s="10" t="inlineStr">
         <is>
-          <t>卖出</t>
+          <t>买入</t>
         </is>
       </c>
       <c r="C19" s="10" t="n">
-        <v>1.1458</v>
+        <v>1</v>
       </c>
       <c r="D19" s="10" t="n">
-        <v>353.3514</v>
+        <v>396.27</v>
       </c>
       <c r="E19" s="10" t="n">
         <v>0</v>
@@ -1034,7 +1034,7 @@
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
         <is>
-          <t>2025-12-23</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B20" s="10" t="inlineStr">
@@ -1046,7 +1046,7 @@
         <v>1</v>
       </c>
       <c r="D20" s="10" t="n">
-        <v>349.5</v>
+        <v>398.6828</v>
       </c>
       <c r="E20" s="10" t="n">
         <v>0</v>
@@ -1071,7 +1071,7 @@
     <row r="21">
       <c r="A21" s="9" t="inlineStr">
         <is>
-          <t>2025-12-23</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B21" s="10" t="inlineStr">
@@ -1080,10 +1080,10 @@
         </is>
       </c>
       <c r="C21" s="10" t="n">
-        <v>0.0723</v>
+        <v>5</v>
       </c>
       <c r="D21" s="10" t="n">
-        <v>345.7</v>
+        <v>401.385</v>
       </c>
       <c r="E21" s="10" t="n">
         <v>0</v>
@@ -1108,46 +1108,60 @@
     <row r="22">
       <c r="A22" s="9" t="inlineStr">
         <is>
-          <t>2025-12-22</t>
+          <t>2026-01-02</t>
         </is>
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>买入</t>
+          <t>卖出</t>
         </is>
       </c>
       <c r="C22" s="10" t="n">
-        <v>0.0735</v>
+        <v>1.1458</v>
       </c>
       <c r="D22" s="10" t="n">
-        <v>340.0563</v>
+        <v>353.3514</v>
       </c>
       <c r="E22" s="10" t="n">
         <v>0</v>
       </c>
       <c r="F22" s="11">
-        <f>IF(B22="卖出",(D22-G22)*C22-E22,"")</f>
+        <f>IF(B22="卖出",IF(H23&lt;=0,"",(D22-G23)*C22-E22),"")</f>
         <v/>
       </c>
       <c r="G22" s="11">
-        <f>IF(B22="买入",(C22*D22+E22)/C22,"")</f>
+        <f>IF(B22="买入",IF(H23&lt;=0,(C22*D22+E22)/C22,(G23*H23+C22*D22+E22)/(H23+C22)),IF(B22="卖出",IF(H23-C22&lt;=0,G23,(G23*H23-C22*D22+E22)/(H23-C22)),""))</f>
         <v/>
       </c>
       <c r="H22" s="11">
-        <f>IF(B22="买入",C22,IF(B22="卖出",-C22,""))</f>
+        <f>IF(B22="买入",H23+C22,IF(B22="卖出",MAX(0,H23-C22),""))</f>
         <v/>
       </c>
       <c r="I22">
-        <f>IF(B22="买入",0,IF(B22="卖出",IF(H22=0,0,F22),0))</f>
+        <f>IF(B22="",I23,IF(B22="买入",I23,IF(B22="卖出",IF(H22=0,0,I23+F22),I23)))</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="9" t="n"/>
-      <c r="B23" s="10" t="n"/>
-      <c r="C23" s="10" t="n"/>
-      <c r="D23" s="10" t="n"/>
-      <c r="E23" s="10" t="n"/>
+      <c r="A23" s="9" t="inlineStr">
+        <is>
+          <t>2025-12-23</t>
+        </is>
+      </c>
+      <c r="B23" s="10" t="inlineStr">
+        <is>
+          <t>买入</t>
+        </is>
+      </c>
+      <c r="C23" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" s="10" t="n">
+        <v>349.5</v>
+      </c>
+      <c r="E23" s="10" t="n">
+        <v>0</v>
+      </c>
       <c r="F23" s="11">
         <f>IF(B23="卖出",IF(H24&lt;=0,"",(D23-G24)*C23-E23),"")</f>
         <v/>
@@ -1166,11 +1180,25 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="9" t="n"/>
-      <c r="B24" s="10" t="n"/>
-      <c r="C24" s="10" t="n"/>
-      <c r="D24" s="10" t="n"/>
-      <c r="E24" s="10" t="n"/>
+      <c r="A24" s="9" t="inlineStr">
+        <is>
+          <t>2025-12-23</t>
+        </is>
+      </c>
+      <c r="B24" s="10" t="inlineStr">
+        <is>
+          <t>买入</t>
+        </is>
+      </c>
+      <c r="C24" s="10" t="n">
+        <v>0.0723</v>
+      </c>
+      <c r="D24" s="10" t="n">
+        <v>345.7</v>
+      </c>
+      <c r="E24" s="10" t="n">
+        <v>0</v>
+      </c>
       <c r="F24" s="11">
         <f>IF(B24="卖出",IF(H25&lt;=0,"",(D24-G25)*C24-E24),"")</f>
         <v/>
@@ -1189,25 +1217,39 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="9" t="n"/>
-      <c r="B25" s="10" t="n"/>
-      <c r="C25" s="10" t="n"/>
-      <c r="D25" s="10" t="n"/>
-      <c r="E25" s="10" t="n"/>
+      <c r="A25" s="9" t="inlineStr">
+        <is>
+          <t>2025-12-22</t>
+        </is>
+      </c>
+      <c r="B25" s="10" t="inlineStr">
+        <is>
+          <t>买入</t>
+        </is>
+      </c>
+      <c r="C25" s="10" t="n">
+        <v>0.0735</v>
+      </c>
+      <c r="D25" s="10" t="n">
+        <v>340.0563</v>
+      </c>
+      <c r="E25" s="10" t="n">
+        <v>0</v>
+      </c>
       <c r="F25" s="11">
-        <f>IF(B25="卖出",IF(H26&lt;=0,"",(D25-G26)*C25-E25),"")</f>
+        <f>IF(B25="卖出",(D25-G25)*C25-E25,"")</f>
         <v/>
       </c>
       <c r="G25" s="11">
-        <f>IF(B25="买入",IF(H26&lt;=0,(C25*D25+E25)/C25,(G26*H26+C25*D25+E25)/(H26+C25)),IF(B25="卖出",IF(H26-C25&lt;=0,G26,(G26*H26-C25*D25+E25)/(H26-C25)),""))</f>
+        <f>IF(B25="买入",(C25*D25+E25)/C25,"")</f>
         <v/>
       </c>
       <c r="H25" s="11">
-        <f>IF(B25="买入",H26+C25,IF(B25="卖出",MAX(0,H26-C25),""))</f>
+        <f>IF(B25="买入",C25,IF(B25="卖出",-C25,""))</f>
         <v/>
       </c>
       <c r="I25">
-        <f>IF(B25="",I26,IF(B25="买入",I26,IF(B25="卖出",IF(H25=0,0,I26+F25),I26)))</f>
+        <f>IF(B25="买入",0,IF(B25="卖出",IF(H25=0,0,F25),0))</f>
         <v/>
       </c>
     </row>
@@ -3132,7 +3174,7 @@
     </row>
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="7">
-        <f>IF(COUNTA(B10:B104)=0,"","⚖️ 盈亏平衡点: $"&amp;TEXT(G10-I10/H10,"#,##0.00"))</f>
+        <f>IF(COUNTA(B10:B104)=0,"","⚖️ 盈亏平衡点: $"&amp;TEXT(G10-IFERROR(I10/H10,0),"#,##0.00")&amp;"  (差价: $"&amp;TEXT(-IFERROR(I10/H10,0),"#,##0.00")&amp;")")</f>
         <v/>
       </c>
     </row>
@@ -5481,7 +5523,7 @@
     </row>
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="7">
-        <f>IF(COUNTA(B10:B104)=0,"","⚖️ 盈亏平衡点: $"&amp;TEXT(G10-I10/H10,"#,##0.00"))</f>
+        <f>IF(COUNTA(B10:B104)=0,"","⚖️ 盈亏平衡点: $"&amp;TEXT(G10-IFERROR(I10/H10,0),"#,##0.00")&amp;"  (差价: $"&amp;TEXT(-IFERROR(I10/H10,0),"#,##0.00")&amp;")")</f>
         <v/>
       </c>
     </row>
@@ -7830,7 +7872,7 @@
     </row>
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="7">
-        <f>IF(COUNTA(B10:B104)=0,"","⚖️ 盈亏平衡点: $"&amp;TEXT(G10-I10/H10,"#,##0.00"))</f>
+        <f>IF(COUNTA(B10:B104)=0,"","⚖️ 盈亏平衡点: $"&amp;TEXT(G10-IFERROR(I10/H10,0),"#,##0.00")&amp;"  (差价: $"&amp;TEXT(-IFERROR(I10/H10,0),"#,##0.00")&amp;")")</f>
         <v/>
       </c>
     </row>
@@ -10179,7 +10221,7 @@
     </row>
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="7">
-        <f>IF(COUNTA(B10:B104)=0,"","⚖️ 盈亏平衡点: $"&amp;TEXT(G10-I10/H10,"#,##0.00"))</f>
+        <f>IF(COUNTA(B10:B104)=0,"","⚖️ 盈亏平衡点: $"&amp;TEXT(G10-IFERROR(I10/H10,0),"#,##0.00")&amp;"  (差价: $"&amp;TEXT(-IFERROR(I10/H10,0),"#,##0.00")&amp;")")</f>
         <v/>
       </c>
     </row>
@@ -12808,7 +12850,7 @@
     </row>
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="7">
-        <f>IF(COUNTA(B10:B104)=0,"","⚖️ 盈亏平衡点: $"&amp;TEXT(G10-I10/H10,"#,##0.00"))</f>
+        <f>IF(COUNTA(B10:B104)=0,"","⚖️ 盈亏平衡点: $"&amp;TEXT(G10-IFERROR(I10/H10,0),"#,##0.00")&amp;"  (差价: $"&amp;TEXT(-IFERROR(I10/H10,0),"#,##0.00")&amp;")")</f>
         <v/>
       </c>
     </row>

</xml_diff>